<commit_message>
feat(tools): dashboard com radar e formulas COUNTIF
</commit_message>
<xml_diff>
--- a/templates/avaliacao-maturidade-qnrcs.xlsx
+++ b/templates/avaliacao-maturidade-qnrcs.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DE" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RS" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RC" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -53,7 +54,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -68,6 +69,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -97,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -121,6 +127,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -220,6 +238,122 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <style val="26"/>
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Perfil de maturidade por objectivo</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <radarChart>
+        <radarStyle val="filled"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Dashboard'!F3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Dashboard'!$A$4:$A$9</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Dashboard'!$F$4:$F$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </radarChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>12</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5760000" cy="4320000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1903,4 +2037,260 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F33"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Dashboard — Perfil de maturidade QNRCS v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Objectivo</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Sim</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Não</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>% Maturidade</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Gerir</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="C4" s="6">
+        <f>COUNTIF('GR'!C3:C8,"Sim")</f>
+        <v/>
+      </c>
+      <c r="D4" s="6">
+        <f>COUNTIF('GR'!C3:C8,"Parcial")</f>
+        <v/>
+      </c>
+      <c r="E4" s="6">
+        <f>COUNTIF('GR'!C3:C8,"Não")</f>
+        <v/>
+      </c>
+      <c r="F4" s="9">
+        <f>(C4*1+D4*0.5)/B4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Identificar</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C5" s="6">
+        <f>COUNTIF('ID'!C3:C6,"Sim")</f>
+        <v/>
+      </c>
+      <c r="D5" s="6">
+        <f>COUNTIF('ID'!C3:C6,"Parcial")</f>
+        <v/>
+      </c>
+      <c r="E5" s="6">
+        <f>COUNTIF('ID'!C3:C6,"Não")</f>
+        <v/>
+      </c>
+      <c r="F5" s="9">
+        <f>(C5*1+D5*0.5)/B5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Proteger</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" s="6">
+        <f>COUNTIF('PR'!C3:C9,"Sim")</f>
+        <v/>
+      </c>
+      <c r="D6" s="6">
+        <f>COUNTIF('PR'!C3:C9,"Parcial")</f>
+        <v/>
+      </c>
+      <c r="E6" s="6">
+        <f>COUNTIF('PR'!C3:C9,"Não")</f>
+        <v/>
+      </c>
+      <c r="F6" s="9">
+        <f>(C6*1+D6*0.5)/B6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Detectar</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="6">
+        <f>COUNTIF('DE'!C3:C5,"Sim")</f>
+        <v/>
+      </c>
+      <c r="D7" s="6">
+        <f>COUNTIF('DE'!C3:C5,"Parcial")</f>
+        <v/>
+      </c>
+      <c r="E7" s="6">
+        <f>COUNTIF('DE'!C3:C5,"Não")</f>
+        <v/>
+      </c>
+      <c r="F7" s="9">
+        <f>(C7*1+D7*0.5)/B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>Responder</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C8" s="6">
+        <f>COUNTIF('RS'!C3:C6,"Sim")</f>
+        <v/>
+      </c>
+      <c r="D8" s="6">
+        <f>COUNTIF('RS'!C3:C6,"Parcial")</f>
+        <v/>
+      </c>
+      <c r="E8" s="6">
+        <f>COUNTIF('RS'!C3:C6,"Não")</f>
+        <v/>
+      </c>
+      <c r="F8" s="9">
+        <f>(C8*1+D8*0.5)/B8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Recuperar</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C9" s="6">
+        <f>COUNTIF('RC'!C3:C4,"Sim")</f>
+        <v/>
+      </c>
+      <c r="D9" s="6">
+        <f>COUNTIF('RC'!C3:C4,"Parcial")</f>
+        <v/>
+      </c>
+      <c r="E9" s="6">
+        <f>COUNTIF('RC'!C3:C4,"Não")</f>
+        <v/>
+      </c>
+      <c r="F9" s="9">
+        <f>(C9*1+D9*0.5)/B9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B10" s="10">
+        <f>SUM(B4:B9)</f>
+        <v/>
+      </c>
+      <c r="C10" s="10">
+        <f>SUM(C4:C9)</f>
+        <v/>
+      </c>
+      <c r="D10" s="10">
+        <f>SUM(D4:D9)</f>
+        <v/>
+      </c>
+      <c r="E10" s="10">
+        <f>SUM(E4:E9)</f>
+        <v/>
+      </c>
+      <c r="F10" s="11">
+        <f>(C10*1+D10*0.5)/B10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33" ht="60" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>Os objectivos com pontuação mais baixa são candidatos prioritários para o roadmap E.3 dos próximos 6 meses. Reveja em cada aba os controlos marcados como 'Não' ou 'Parcial' e priorize os com Mapeamento Anexo IV (coluna E).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>